<commit_message>
New code for polarization
</commit_message>
<xml_diff>
--- a/LinMeas/Fiber/PulledDatFiber.xlsx
+++ b/LinMeas/Fiber/PulledDatFiber.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\LinMeas\Fiber\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECFB2911-113A-44EF-837C-210AB94C945D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661F4232-520F-4D99-B22C-6FD27DBB31EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PulledDat" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t>lin</t>
   </si>
@@ -49,6 +50,15 @@
   </si>
   <si>
     <t>Hot cell PD</t>
+  </si>
+  <si>
+    <t>Hot</t>
+  </si>
+  <si>
+    <t>Long</t>
+  </si>
+  <si>
+    <t>Pwr</t>
   </si>
 </sst>
 </file>
@@ -5323,15 +5333,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>500062</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>233362</xdr:colOff>
+      <xdr:row>28</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -5360,15 +5370,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>85724</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>104776</xdr:rowOff>
+      <xdr:colOff>400049</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>133351</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5733,10 +5743,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1">
         <v>5.5241300000000004</v>
       </c>
@@ -5780,7 +5790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>4.4030699999999996</v>
       </c>
@@ -5836,7 +5846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3.677</v>
       </c>
@@ -5903,8 +5913,17 @@
         <f>X3/W3*100</f>
         <v>0.11104941699056081</v>
       </c>
+      <c r="AB3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>6</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3.2809200000000001</v>
       </c>
@@ -5971,8 +5990,11 @@
         <f t="shared" ref="Y4:Y35" si="5">X4/W4*100</f>
         <v>0.22209883398112162</v>
       </c>
+      <c r="AA4" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2.91757</v>
       </c>
@@ -6039,8 +6061,11 @@
         <f t="shared" si="5"/>
         <v>0.33314825097168238</v>
       </c>
+      <c r="AA5" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2.4418199999999999</v>
       </c>
@@ -6107,8 +6132,11 @@
         <f t="shared" si="5"/>
         <v>0.44419766796224325</v>
       </c>
+      <c r="AA6" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2.2521900000000001</v>
       </c>
@@ -6176,7 +6204,7 @@
         <v>0.55524708495280395</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2.01783</v>
       </c>
@@ -6244,7 +6272,7 @@
         <v>0.66629650194336476</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1.76278</v>
       </c>
@@ -6312,7 +6340,7 @@
         <v>0.77734591893392568</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1.4788699999999999</v>
       </c>
@@ -6380,7 +6408,7 @@
         <v>0.8883953359244865</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1.2344299999999999</v>
       </c>
@@ -6448,7 +6476,7 @@
         <v>0.9994447529150472</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0.97243999999999997</v>
       </c>
@@ -6516,7 +6544,7 @@
         <v>1.1104941699056079</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>0.87726999999999999</v>
       </c>
@@ -6584,7 +6612,7 @@
         <v>1.2215435868961688</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0.58377999999999997</v>
       </c>
@@ -6652,7 +6680,7 @@
         <v>1.3325930038867295</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0.41416999999999998</v>
       </c>
@@ -6720,7 +6748,7 @@
         <v>1.4436424208772902</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>0.29103000000000001</v>
       </c>
@@ -7836,4 +7864,13 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFC07CAF-1DF3-4C7F-9C00-960D72354AD5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>